<commit_message>
Update testing levels and types tables
</commit_message>
<xml_diff>
--- a/docs/sprint2/test-plan-tables.xlsx
+++ b/docs/sprint2/test-plan-tables.xlsx
@@ -668,9 +668,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -720,7 +720,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -912,8 +912,8 @@
       <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
+      <c r="F2" s="1" t="str">
+        <v>Так, спринт 4 після отримання модуля</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>13</v>
@@ -935,8 +935,8 @@
       <c r="E3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>18</v>
+      <c r="F3" s="1" t="str">
+        <v>Так, після отримання модуля й модульних тестів</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>13</v>
@@ -1004,8 +1004,8 @@
       <c r="E6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>36</v>
+      <c r="F6" s="1" t="str">
+        <v>Так: на demo після системного; нова функція — після стенда</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>37</v>
@@ -1027,8 +1027,8 @@
       <c r="E7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>43</v>
+      <c r="F7" s="1" t="str">
+        <v>Так, після появи окремого стенда й нової функції</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>44</v>
@@ -1050,8 +1050,8 @@
       <c r="E8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>49</v>
+      <c r="F8" s="1" t="str">
+        <v>Так, після реалізації функції та появи стенда</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>50</v>
@@ -1173,37 +1173,37 @@
       <c r="A5" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>56</v>
+      <c r="B5" s="1" t="str">
+        <v>Так, частково; серверна частина — після стенда</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>76</v>
+      <c r="D5" s="1" t="str">
+        <v>На demo перевірити прямий URL Profile без входу та відсутність пароля в URL під час звичайного входу. Перевірки блокування після 5 помилок входу та серверних обмежень виконати лише на ізольованому стенді; до його появи вони заблоковані.</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>79</v>
+      <c r="F5" s="1" t="str">
+        <v>Demo, DevTools; ізольований стенд і тестові логіни для серверних перевірок</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <v>Гостьовий доступ доступний для перевірки зараз; активні серверні перевірки очікують стенда.</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="96.95" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>56</v>
+      <c r="B6" s="1" t="str">
+        <v>Так, частково; повний потік — після стенда</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>82</v>
+      <c r="D6" s="1" t="str">
+        <v>На demo зіставити власний коментар і відносну зміну Votes після голосу. Після отримання модуля перевірити VoteValidator → RatingAggregator на фікстурах; наскрізний шлях із записом у БД — лише після появи окремого стенда.</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>83</v>
@@ -1211,31 +1211,31 @@
       <c r="F6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>85</v>
+      <c r="G6" s="1" t="str">
+        <v>UI-потік доступний на demo; серверний запис і агрегація потребують контрольованого середовища.</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="96.95" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>56</v>
+      <c r="B7" s="1" t="str">
+        <v>Так, частково; негативні API-кейси — після стенда</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>88</v>
+      <c r="D7" s="1" t="str">
+        <v>На demo спостерігати через DevTools Network відповіді звичайних ручних дій: HTTP status і поля JSON моделей/голосів. Прямі негативні API-запити, змінені дані й серверні помилки — лише після отримання дозволеного стенда.</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>91</v>
+      <c r="F7" s="1" t="str">
+        <v>Chrome DevTools Network, JSON; окремий стенд для негативних API-кейсів</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <v>Пасивне спостереження доступне зараз; активні API-перевірки заблоковані до появи стенда.</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="96.95" customHeight="1">
@@ -1288,46 +1288,46 @@
       <c r="A10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>56</v>
+      <c r="B10" s="1" t="str">
+        <v>Так; модуль — після отримання, UI — після стенда</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>104</v>
+      <c r="D10" s="1" t="str">
+        <v>Після отримання autorate-module перевірити сортування 1, 5, 6 і 1000 CarModel у JUnit. Генерацію каталогу в БД та перевірку кількості сторінок виконати після появи власного стенда; на demo чужий каталог не змінювати.</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>107</v>
+      <c r="F10" s="1" t="str">
+        <v>Фікстури CarModel, JUnit 5; окремий вебстенд для пагінації</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <v>Модульний обсяг не потребує вебстенда; UI з контрольованими розмірами каталогу зараз заблокований.</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="96.95" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>56</v>
+      <c r="B11" s="1" t="str">
+        <v>Так, частково; збої — після стенда</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>110</v>
+      <c r="D11" s="1" t="str">
+        <v>На demo після власного голосу оновити сторінку й повторно ввійти: коментар залишається, повторний голос недоступний. Імітацію збоїв запису та перевірку журналів виконати після появи ізольованого стенда.</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>113</v>
+      <c r="F11" s="1" t="str">
+        <v>Chrome/Firefox, власні тестові логіни; ізольований стенд і журнали для збоїв</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <v>Збереження результату після оновлення доступне зараз; керовані збої очікують стенда.</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="96.95" customHeight="1">
@@ -1346,10 +1346,12 @@
       <c r="E12" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G12" s="1"/>
+      <c r="F12" s="1" t="str">
+        <v>—</v>
+      </c>
+      <c r="G12" s="1" t="str">
+        <v>Немає вимоги або доступної архітектури резервування/гарячої заміни вузлів; звичайна доступність сторінок перевіряється smoke.</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="96.95" customHeight="1">
       <c r="A13" s="1" t="s">
@@ -1367,10 +1369,12 @@
       <c r="E13" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G13" s="1"/>
+      <c r="F13" s="1" t="str">
+        <v>—</v>
+      </c>
+      <c r="G13" s="1" t="str">
+        <v>Система не має у вимогах резервних вузлів і сценарію перемикання після їх відмови; відновлення окремого браузерного сеансу входить у надійність.</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="96.95" customHeight="1">
       <c r="A14" s="1" t="s">
@@ -1411,10 +1415,12 @@
       <c r="E15" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="G15" s="1"/>
+      <c r="F15" s="1" t="str">
+        <v>—</v>
+      </c>
+      <c r="G15" s="1" t="str">
+        <v>Єдина мова UI за SRS — англійська, окремої перекладеної версії продукту немає; Unicode-коментарі перевіряє i18n.</v>
+      </c>
     </row>
     <row r="16" spans="1:7" ht="96.95" customHeight="1">
       <c r="A16" s="1" t="s">
@@ -1443,8 +1449,8 @@
       <c r="A17" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>56</v>
+      <c r="B17" s="1" t="str">
+        <v>Так, заблоковано до появи стенда</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>133</v>
@@ -1458,16 +1464,16 @@
       <c r="F17" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>137</v>
+      <c r="G17" s="1" t="str">
+        <v>Виконання після отримання ізольованого стенда, тестової БД і дозволу на навантаження. На demo не запускається.</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="96.95" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>56</v>
+      <c r="B18" s="1" t="str">
+        <v>Так, заблоковано до появи стенда</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>139</v>
@@ -1481,16 +1487,16 @@
       <c r="F18" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>143</v>
+      <c r="G18" s="1" t="str">
+        <v>Виконання після розгортання ізольованого стенда й БД та погодження меж навантаження. На demo не запускається.</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="96.95" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>56</v>
+      <c r="B19" s="1" t="str">
+        <v>Так, заблоковано до появи стенда</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>145</v>
@@ -1504,8 +1510,8 @@
       <c r="F19" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>149</v>
+      <c r="G19" s="1" t="str">
+        <v>Виконання після розгортання ізольованого стенда й погодження навантаження. На demo не запускається.</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="96.95" customHeight="1">
@@ -1558,23 +1564,23 @@
       <c r="A22" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>56</v>
+      <c r="B22" s="1" t="str">
+        <v>Так, після отримання модуля</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>164</v>
+      <c r="D22" s="1" t="str">
+        <v>Після отримання autorate-module у тестовій JVM 1 год повторювати ModelSearch.search і RatingAggregator.topN на однакових фікстурах; порівняти перші й останні 10 хв.</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>167</v>
+      <c r="F22" s="1" t="str">
+        <v>JFR, метрики JVM, autorate-module</v>
+      </c>
+      <c r="G22" s="1" t="str">
+        <v>Модульна перевірка не потребує повного вебстенда; очікує отримання вихідного модуля.</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="96.95" customHeight="1">
@@ -1604,8 +1610,8 @@
       <c r="A24" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>56</v>
+      <c r="B24" s="1" t="str">
+        <v>Так, заблоковано до появи стенда</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>175</v>
@@ -1619,31 +1625,31 @@
       <c r="F24" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>179</v>
+      <c r="G24" s="1" t="str">
+        <v>Повний шлях із записом у БД заблокований до появи контрольованого стенда; профілювання самого модуля виконується окремо.</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="96.95" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>56</v>
+      <c r="B25" s="1" t="str">
+        <v>Так, High; заблоковано до появи API/БД</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>182</v>
+      <c r="D25" s="1" t="str">
+        <v>Після отримання ізольованого API та БД синхронно надіслати через бар’єр потоків 2 vote з однаковою парою userId/modelId; перевірити рівно 1 збережений голос і 1 відмову. До появи стенда виконання заблоковане. Послідовний тест BL-30 перевіряє дубль, але не доводить атомарності запису.</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>185</v>
+      <c r="F25" s="1" t="str">
+        <v>JUnit concurrency, бар’єр потоків, ізольовані API та БД</v>
+      </c>
+      <c r="G25" s="1" t="str">
+        <v>Критичний пріоритет High (порядок 4). Повторити перед релізом; відсутність стенда залишає перевірку заблокованою.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>